<commit_message>
Fix incorrect werkloosheidsgraad values for Globe, Vossegat, Sint-Denijs (2022-2023)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data Brussels Neighborhoods v2.xlsx
+++ b/Data Brussels Neighborhoods v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cursist\Desktop\FARI\MapVizApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA75CD68-CCCA-4110-B1D8-C28C8283887C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E525C5C-5041-4456-B30E-549B16765803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -102348,10 +102348,10 @@
         <v>13.98</v>
       </c>
       <c r="HY59">
-        <v>64.8</v>
+        <v>13.98</v>
       </c>
       <c r="HZ59">
-        <v>83.94</v>
+        <v>13.98</v>
       </c>
       <c r="IA59">
         <v>24</v>
@@ -104099,10 +104099,10 @@
         <v>14.4</v>
       </c>
       <c r="HY60">
-        <v>51.8</v>
+        <v>14.4</v>
       </c>
       <c r="HZ60">
-        <v>75.53</v>
+        <v>14.4</v>
       </c>
       <c r="IA60">
         <v>30.6</v>
@@ -105850,10 +105850,10 @@
         <v>21.04</v>
       </c>
       <c r="HY61">
-        <v>68.599999999999994</v>
+        <v>21.04</v>
       </c>
       <c r="HZ61">
-        <v>97.82</v>
+        <v>21.04</v>
       </c>
       <c r="IA61">
         <v>19.899999999999999</v>

</xml_diff>

<commit_message>
Update Excel data and regenerate data files
Commit updated Excel file and regenerated JSON/GeoJSON data
(58 neighborhoods, 39 indicators, 1981-2025).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data Brussels Neighborhoods v2.xlsx
+++ b/Data Brussels Neighborhoods v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cursist\Desktop\FARI\MapVizApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E525C5C-5041-4456-B30E-549B16765803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F2D587-661D-4231-B535-357CE501FD0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -471,7 +471,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -486,6 +486,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1A1A2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -510,7 +516,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -530,21 +536,19 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -876,7 +880,6 @@
   <dimension ref="A1:WK67"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.5546875" bestFit="1" customWidth="1"/>
     <col min="581" max="585" width="22" customWidth="1"/>
   </cols>
@@ -6012,8 +6015,8 @@
       </c>
     </row>
     <row r="4" spans="1:609" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>2</v>
+      <c r="A4" s="10">
+        <v>8</v>
       </c>
       <c r="B4" t="s">
         <v>46</v>
@@ -7752,25 +7755,25 @@
       <c r="VH4">
         <v>13.33</v>
       </c>
-      <c r="VI4" s="3">
-        <v>100</v>
+      <c r="VI4" s="5">
+        <v>56</v>
       </c>
       <c r="VJ4" s="4">
-        <v>92.8</v>
+        <v>48</v>
       </c>
       <c r="VK4" s="4">
-        <v>65.8</v>
+        <v>21.2</v>
       </c>
       <c r="VL4" s="4">
-        <v>69</v>
+        <v>64.3</v>
       </c>
       <c r="VM4" s="4">
-        <v>57</v>
+        <v>76.2</v>
       </c>
     </row>
     <row r="5" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
         <v>47</v>
@@ -9510,24 +9513,24 @@
         <v>11.54</v>
       </c>
       <c r="VI5" s="5">
-        <v>49.9</v>
+        <v>60.9</v>
       </c>
       <c r="VJ5" s="4">
-        <v>40.700000000000003</v>
+        <v>46.3</v>
       </c>
       <c r="VK5" s="4">
-        <v>9.1999999999999993</v>
+        <v>29</v>
       </c>
       <c r="VL5" s="4">
-        <v>54.8</v>
+        <v>68.3</v>
       </c>
       <c r="VM5" s="4">
-        <v>95.3</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
         <v>49</v>
@@ -11266,25 +11269,25 @@
       <c r="VH6">
         <v>18.77</v>
       </c>
-      <c r="VI6" s="5">
-        <v>54.2</v>
+      <c r="VI6" s="3">
+        <v>100</v>
       </c>
       <c r="VJ6" s="4">
-        <v>46.7</v>
+        <v>92.8</v>
       </c>
       <c r="VK6" s="4">
-        <v>16.399999999999999</v>
+        <v>65.8</v>
       </c>
       <c r="VL6" s="4">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="VM6" s="4">
-        <v>93.1</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
         <v>51</v>
@@ -13023,25 +13026,25 @@
       <c r="VH7">
         <v>25.73</v>
       </c>
-      <c r="VI7" s="5">
-        <v>52.6</v>
+      <c r="VI7" s="3">
+        <v>80.8</v>
       </c>
       <c r="VJ7" s="4">
-        <v>41.6</v>
+        <v>59</v>
       </c>
       <c r="VK7" s="4">
-        <v>28.4</v>
+        <v>47.3</v>
       </c>
       <c r="VL7" s="4">
-        <v>47.7</v>
+        <v>71.7</v>
       </c>
       <c r="VM7" s="4">
-        <v>90.1</v>
+        <v>81.2</v>
       </c>
     </row>
     <row r="8" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
         <v>52</v>
@@ -14780,25 +14783,25 @@
       <c r="VH8">
         <v>12.78</v>
       </c>
-      <c r="VI8" s="5">
-        <v>42.3</v>
+      <c r="VI8" s="3">
+        <v>86.3</v>
       </c>
       <c r="VJ8" s="4">
-        <v>18.7</v>
+        <v>72.5</v>
       </c>
       <c r="VK8" s="4">
-        <v>37.5</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="VL8" s="4">
-        <v>48.7</v>
+        <v>69.3</v>
       </c>
       <c r="VM8" s="4">
-        <v>93.4</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="9" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
         <v>53</v>
@@ -16537,25 +16540,25 @@
       <c r="VH9">
         <v>12.7</v>
       </c>
-      <c r="VI9" s="6">
-        <v>28.5</v>
+      <c r="VI9" s="3">
+        <v>89.4</v>
       </c>
       <c r="VJ9" s="4">
-        <v>24.3</v>
+        <v>85.4</v>
       </c>
       <c r="VK9" s="4">
-        <v>2.6</v>
+        <v>31.3</v>
       </c>
       <c r="VL9" s="4">
-        <v>44.8</v>
+        <v>66.8</v>
       </c>
       <c r="VM9" s="4">
-        <v>91.1</v>
+        <v>79.099999999999994</v>
       </c>
     </row>
     <row r="10" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
         <v>54</v>
@@ -18294,25 +18297,25 @@
       <c r="VH10">
         <v>16.489999999999998</v>
       </c>
-      <c r="VI10" s="5">
-        <v>48.2</v>
+      <c r="VI10" s="3">
+        <v>76.400000000000006</v>
       </c>
       <c r="VJ10" s="4">
-        <v>40</v>
+        <v>79.5</v>
       </c>
       <c r="VK10" s="4">
-        <v>8.8000000000000007</v>
+        <v>48.1</v>
       </c>
       <c r="VL10" s="4">
-        <v>55.4</v>
+        <v>59.5</v>
       </c>
       <c r="VM10" s="4">
-        <v>92.5</v>
+        <v>53.2</v>
       </c>
     </row>
     <row r="11" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
         <v>55</v>
@@ -20051,25 +20054,25 @@
       <c r="VH11">
         <v>10.48</v>
       </c>
-      <c r="VI11" s="6">
-        <v>31.5</v>
+      <c r="VI11" s="3">
+        <v>77.2</v>
       </c>
       <c r="VJ11" s="4">
-        <v>18.5</v>
+        <v>94.7</v>
       </c>
       <c r="VK11" s="4">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="VL11" s="4">
-        <v>52.8</v>
+        <v>57.2</v>
       </c>
       <c r="VM11" s="4">
-        <v>100</v>
+        <v>55.1</v>
       </c>
     </row>
     <row r="12" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
         <v>56</v>
@@ -21808,25 +21811,25 @@
       <c r="VH12">
         <v>11.26</v>
       </c>
-      <c r="VI12" s="6">
-        <v>30</v>
+      <c r="VI12" s="3">
+        <v>85.5</v>
       </c>
       <c r="VJ12" s="4">
-        <v>20.5</v>
+        <v>85</v>
       </c>
       <c r="VK12" s="4">
-        <v>12.1</v>
+        <v>25.4</v>
       </c>
       <c r="VL12" s="4">
-        <v>40</v>
+        <v>61.9</v>
       </c>
       <c r="VM12" s="4">
-        <v>96.8</v>
+        <v>81.900000000000006</v>
       </c>
     </row>
     <row r="13" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
         <v>57</v>
@@ -23565,25 +23568,25 @@
       <c r="VH13">
         <v>13.61</v>
       </c>
-      <c r="VI13" s="5">
-        <v>57.5</v>
+      <c r="VI13" s="3">
+        <v>82.4</v>
       </c>
       <c r="VJ13" s="4">
-        <v>22.8</v>
+        <v>100</v>
       </c>
       <c r="VK13" s="4">
-        <v>79.099999999999994</v>
+        <v>26.2</v>
       </c>
       <c r="VL13" s="4">
-        <v>35.6</v>
+        <v>56</v>
       </c>
       <c r="VM13" s="4">
-        <v>95.7</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="14" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
         <v>58</v>
@@ -25322,25 +25325,25 @@
       <c r="VH14">
         <v>13.99</v>
       </c>
-      <c r="VI14" s="5">
-        <v>45.3</v>
+      <c r="VI14" s="3">
+        <v>89.5</v>
       </c>
       <c r="VJ14" s="4">
-        <v>36.9</v>
+        <v>96.6</v>
       </c>
       <c r="VK14" s="4">
-        <v>30.5</v>
+        <v>38.5</v>
       </c>
       <c r="VL14" s="4">
-        <v>43.1</v>
+        <v>60.6</v>
       </c>
       <c r="VM14" s="4">
-        <v>84.4</v>
+        <v>62.4</v>
       </c>
     </row>
     <row r="15" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
         <v>59</v>
@@ -27080,24 +27083,24 @@
         <v>17.940000000000001</v>
       </c>
       <c r="VI15" s="5">
-        <v>48</v>
+        <v>63.2</v>
       </c>
       <c r="VJ15" s="4">
-        <v>26</v>
+        <v>67.900000000000006</v>
       </c>
       <c r="VK15" s="4">
-        <v>53.1</v>
+        <v>31.5</v>
       </c>
       <c r="VL15" s="4">
-        <v>37.700000000000003</v>
+        <v>55.9</v>
       </c>
       <c r="VM15" s="4">
-        <v>92.2</v>
+        <v>61.2</v>
       </c>
     </row>
     <row r="16" spans="1:609" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s">
         <v>60</v>
@@ -28836,25 +28839,23 @@
       <c r="VH16">
         <v>15</v>
       </c>
-      <c r="VI16" s="5">
-        <v>50.9</v>
-      </c>
+      <c r="VI16" s="7"/>
       <c r="VJ16" s="4">
-        <v>39.799999999999997</v>
+        <v>40.700000000000003</v>
       </c>
       <c r="VK16" s="4">
-        <v>17.399999999999999</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="VL16" s="4">
-        <v>49.8</v>
+        <v>54.8</v>
       </c>
       <c r="VM16" s="4">
-        <v>96.7</v>
+        <v>95.3</v>
       </c>
     </row>
     <row r="17" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
         <v>61</v>
@@ -30593,25 +30594,25 @@
       <c r="VH17">
         <v>15.43</v>
       </c>
-      <c r="VI17" s="3">
-        <v>80.3</v>
+      <c r="VI17" s="5">
+        <v>49.9</v>
       </c>
       <c r="VJ17" s="4">
-        <v>64.2</v>
+        <v>46.7</v>
       </c>
       <c r="VK17" s="4">
-        <v>37.799999999999997</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="VL17" s="4">
-        <v>64.2</v>
+        <v>51</v>
       </c>
       <c r="VM17" s="4">
-        <v>88.7</v>
+        <v>93.1</v>
       </c>
     </row>
     <row r="18" spans="1:585" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="B18" t="s">
         <v>62</v>
@@ -31369,25 +31370,25 @@
       <c r="IS18">
         <v>61.36</v>
       </c>
-      <c r="VI18" s="3">
-        <v>79.8</v>
+      <c r="VI18" s="5">
+        <v>54.2</v>
       </c>
       <c r="VJ18" s="4">
-        <v>78.5</v>
+        <v>41.6</v>
       </c>
       <c r="VK18" s="4">
-        <v>48.6</v>
+        <v>28.4</v>
       </c>
       <c r="VL18" s="4">
-        <v>53.7</v>
+        <v>47.7</v>
       </c>
       <c r="VM18" s="4">
-        <v>67.5</v>
+        <v>90.1</v>
       </c>
     </row>
     <row r="19" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="B19" t="s">
         <v>62</v>
@@ -33127,24 +33128,24 @@
         <v>23.23</v>
       </c>
       <c r="VI19" s="5">
-        <v>68.900000000000006</v>
+        <v>52.6</v>
       </c>
       <c r="VJ19" s="4">
-        <v>65.099999999999994</v>
+        <v>18.7</v>
       </c>
       <c r="VK19" s="4">
-        <v>24.8</v>
+        <v>37.5</v>
       </c>
       <c r="VL19" s="4">
-        <v>62.2</v>
+        <v>48.7</v>
       </c>
       <c r="VM19" s="4">
-        <v>76.8</v>
+        <v>93.4</v>
       </c>
     </row>
     <row r="20" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="B20" t="s">
         <v>64</v>
@@ -34884,24 +34885,24 @@
         <v>21.04</v>
       </c>
       <c r="VI20" s="5">
-        <v>45.9</v>
+        <v>42.3</v>
       </c>
       <c r="VJ20" s="4">
-        <v>42</v>
+        <v>24.3</v>
       </c>
       <c r="VK20" s="4">
-        <v>29.2</v>
+        <v>2.6</v>
       </c>
       <c r="VL20" s="4">
-        <v>44.9</v>
+        <v>44.8</v>
       </c>
       <c r="VM20" s="4">
-        <v>77.400000000000006</v>
+        <v>91.1</v>
       </c>
     </row>
     <row r="21" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>40</v>
+        <v>108</v>
       </c>
       <c r="B21" t="s">
         <v>65</v>
@@ -36641,24 +36642,24 @@
         <v>14.89</v>
       </c>
       <c r="VI21" s="6">
-        <v>18.5</v>
+        <v>28.5</v>
       </c>
       <c r="VJ21" s="4">
-        <v>8.6</v>
+        <v>40</v>
       </c>
       <c r="VK21" s="4">
-        <v>52.7</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="VL21" s="4">
-        <v>12.7</v>
+        <v>55.4</v>
       </c>
       <c r="VM21" s="4">
-        <v>82.8</v>
+        <v>92.5</v>
       </c>
     </row>
     <row r="22" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="B22" t="s">
         <v>66</v>
@@ -38397,25 +38398,25 @@
       <c r="VH22">
         <v>14.25</v>
       </c>
-      <c r="VI22" s="6">
-        <v>27.7</v>
+      <c r="VI22" s="5">
+        <v>48.2</v>
       </c>
       <c r="VJ22" s="4">
-        <v>7.5</v>
+        <v>18.5</v>
       </c>
       <c r="VK22" s="4">
-        <v>79.099999999999994</v>
+        <v>0</v>
       </c>
       <c r="VL22" s="4">
-        <v>19</v>
+        <v>52.8</v>
       </c>
       <c r="VM22" s="4">
-        <v>73.400000000000006</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>42</v>
+        <v>110</v>
       </c>
       <c r="B23" t="s">
         <v>67</v>
@@ -40155,24 +40156,24 @@
         <v>18.41</v>
       </c>
       <c r="VI23" s="6">
-        <v>17.600000000000001</v>
+        <v>31.5</v>
       </c>
       <c r="VJ23" s="4">
-        <v>12.6</v>
+        <v>20.5</v>
       </c>
       <c r="VK23" s="4">
-        <v>65.5</v>
+        <v>12.1</v>
       </c>
       <c r="VL23" s="4">
-        <v>9.3000000000000007</v>
+        <v>40</v>
       </c>
       <c r="VM23" s="4">
-        <v>66.900000000000006</v>
+        <v>96.8</v>
       </c>
     </row>
     <row r="24" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>43</v>
+      <c r="A24" s="10">
+        <v>111</v>
       </c>
       <c r="B24" t="s">
         <v>68</v>
@@ -41912,24 +41913,24 @@
         <v>18.07</v>
       </c>
       <c r="VI24" s="6">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="VJ24" s="4">
-        <v>0</v>
+        <v>22.8</v>
       </c>
       <c r="VK24" s="4">
-        <v>65.7</v>
+        <v>79.099999999999994</v>
       </c>
       <c r="VL24" s="4">
-        <v>0</v>
+        <v>35.6</v>
       </c>
       <c r="VM24" s="4">
-        <v>58</v>
+        <v>95.7</v>
       </c>
     </row>
     <row r="25" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>44</v>
+      <c r="A25" s="10">
+        <v>112</v>
       </c>
       <c r="B25" t="s">
         <v>69</v>
@@ -43668,25 +43669,25 @@
       <c r="VH25">
         <v>29.46</v>
       </c>
-      <c r="VI25" s="6">
-        <v>8.9</v>
+      <c r="VI25" s="5">
+        <v>57.5</v>
       </c>
       <c r="VJ25" s="4">
-        <v>44.3</v>
+        <v>36.9</v>
       </c>
       <c r="VK25" s="4">
-        <v>55.4</v>
+        <v>30.5</v>
       </c>
       <c r="VL25" s="4">
-        <v>2.2000000000000002</v>
+        <v>43.1</v>
       </c>
       <c r="VM25" s="4">
-        <v>17.100000000000001</v>
+        <v>84.4</v>
       </c>
     </row>
     <row r="26" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>45</v>
+        <v>113</v>
       </c>
       <c r="B26" t="s">
         <v>70</v>
@@ -45425,25 +45426,25 @@
       <c r="VH26">
         <v>20.13</v>
       </c>
-      <c r="VI26" s="6">
-        <v>10.199999999999999</v>
+      <c r="VI26" s="5">
+        <v>45.3</v>
       </c>
       <c r="VJ26" s="4">
-        <v>14.2</v>
+        <v>26</v>
       </c>
       <c r="VK26" s="4">
-        <v>44.3</v>
+        <v>53.1</v>
       </c>
       <c r="VL26" s="4">
-        <v>1.9</v>
+        <v>37.700000000000003</v>
       </c>
       <c r="VM26" s="4">
-        <v>75.599999999999994</v>
+        <v>92.2</v>
       </c>
     </row>
     <row r="27" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>46</v>
+        <v>114</v>
       </c>
       <c r="B27" t="s">
         <v>71</v>
@@ -47182,25 +47183,25 @@
       <c r="VH27">
         <v>25.03</v>
       </c>
-      <c r="VI27" s="6">
-        <v>14.8</v>
+      <c r="VI27" s="5">
+        <v>48</v>
       </c>
       <c r="VJ27" s="4">
-        <v>10.6</v>
+        <v>39.799999999999997</v>
       </c>
       <c r="VK27" s="4">
-        <v>46.8</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="VL27" s="4">
-        <v>16.100000000000001</v>
+        <v>49.8</v>
       </c>
       <c r="VM27" s="4">
-        <v>73.599999999999994</v>
+        <v>96.7</v>
       </c>
     </row>
     <row r="28" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>47</v>
+        <v>116</v>
       </c>
       <c r="B28" t="s">
         <v>72</v>
@@ -48940,24 +48941,24 @@
         <v>18.63</v>
       </c>
       <c r="VI28" s="5">
-        <v>58.3</v>
+        <v>50.9</v>
       </c>
       <c r="VJ28" s="4">
-        <v>55</v>
+        <v>64.2</v>
       </c>
       <c r="VK28" s="4">
-        <v>41.4</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="VL28" s="4">
-        <v>99.7</v>
+        <v>64.2</v>
       </c>
       <c r="VM28" s="4">
-        <v>14.7</v>
+        <v>88.7</v>
       </c>
     </row>
     <row r="29" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>48</v>
+        <v>117</v>
       </c>
       <c r="B29" t="s">
         <v>73</v>
@@ -50697,24 +50698,24 @@
         <v>15.71</v>
       </c>
       <c r="VI29" s="3">
-        <v>91.5</v>
+        <v>80.3</v>
       </c>
       <c r="VJ29" s="4">
-        <v>78.599999999999994</v>
+        <v>78.5</v>
       </c>
       <c r="VK29" s="4">
-        <v>80.7</v>
+        <v>48.6</v>
       </c>
       <c r="VL29" s="4">
-        <v>100</v>
+        <v>53.7</v>
       </c>
       <c r="VM29" s="4">
-        <v>14</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="30" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="B30" t="s">
         <v>74</v>
@@ -52453,25 +52454,25 @@
       <c r="VH30">
         <v>14.63</v>
       </c>
-      <c r="VI30" s="5">
-        <v>56</v>
+      <c r="VI30" s="3">
+        <v>79.8</v>
       </c>
       <c r="VJ30" s="4">
-        <v>48</v>
+        <v>65.099999999999994</v>
       </c>
       <c r="VK30" s="4">
-        <v>21.2</v>
+        <v>24.8</v>
       </c>
       <c r="VL30" s="4">
-        <v>64.3</v>
+        <v>62.2</v>
       </c>
       <c r="VM30" s="4">
-        <v>76.2</v>
+        <v>76.8</v>
       </c>
     </row>
     <row r="31" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="B31" t="s">
         <v>75</v>
@@ -54211,24 +54212,24 @@
         <v>14.68</v>
       </c>
       <c r="VI31" s="5">
-        <v>60.9</v>
+        <v>68.900000000000006</v>
       </c>
       <c r="VJ31" s="4">
-        <v>46.3</v>
+        <v>42</v>
       </c>
       <c r="VK31" s="4">
-        <v>29</v>
+        <v>29.2</v>
       </c>
       <c r="VL31" s="4">
-        <v>68.3</v>
+        <v>44.9</v>
       </c>
       <c r="VM31" s="4">
-        <v>78</v>
+        <v>77.400000000000006</v>
       </c>
     </row>
     <row r="32" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A32">
-        <v>51</v>
+      <c r="A32" s="10">
+        <v>9</v>
       </c>
       <c r="B32" t="s">
         <v>76</v>
@@ -55967,25 +55968,25 @@
       <c r="VH32">
         <v>16.760000000000002</v>
       </c>
-      <c r="VI32" s="3">
-        <v>80.8</v>
+      <c r="VI32" s="5">
+        <v>45.9</v>
       </c>
       <c r="VJ32" s="4">
-        <v>59</v>
+        <v>49.6</v>
       </c>
       <c r="VK32" s="4">
-        <v>47.3</v>
+        <v>43</v>
       </c>
       <c r="VL32" s="4">
-        <v>71.7</v>
+        <v>45.1</v>
       </c>
       <c r="VM32" s="4">
-        <v>81.2</v>
+        <v>65.599999999999994</v>
       </c>
     </row>
     <row r="33" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B33" t="s">
         <v>77</v>
@@ -57724,25 +57725,25 @@
       <c r="VH33">
         <v>20.88</v>
       </c>
-      <c r="VI33" s="3">
-        <v>86.3</v>
+      <c r="VI33" s="5">
+        <v>51.7</v>
       </c>
       <c r="VJ33" s="4">
-        <v>72.5</v>
+        <v>45.6</v>
       </c>
       <c r="VK33" s="4">
-        <v>37.799999999999997</v>
+        <v>35.1</v>
       </c>
       <c r="VL33" s="4">
-        <v>69.3</v>
+        <v>55.4</v>
       </c>
       <c r="VM33" s="4">
-        <v>83.5</v>
+        <v>52.7</v>
       </c>
     </row>
     <row r="34" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="B34" t="s">
         <v>78</v>
@@ -59481,25 +59482,25 @@
       <c r="VH34">
         <v>19.7</v>
       </c>
-      <c r="VI34" s="3">
-        <v>89.4</v>
+      <c r="VI34" s="5">
+        <v>44.6</v>
       </c>
       <c r="VJ34" s="4">
-        <v>85.4</v>
+        <v>63.3</v>
       </c>
       <c r="VK34" s="4">
-        <v>31.3</v>
+        <v>100</v>
       </c>
       <c r="VL34" s="4">
-        <v>66.8</v>
+        <v>43</v>
       </c>
       <c r="VM34" s="4">
-        <v>79.099999999999994</v>
+        <v>29.3</v>
       </c>
     </row>
     <row r="35" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A35">
-        <v>54</v>
+      <c r="A35" s="10">
+        <v>12</v>
       </c>
       <c r="B35" t="s">
         <v>79</v>
@@ -61238,25 +61239,25 @@
       <c r="VH35">
         <v>38.369999999999997</v>
       </c>
-      <c r="VI35" s="3">
-        <v>76.400000000000006</v>
+      <c r="VI35" s="5">
+        <v>67.5</v>
       </c>
       <c r="VJ35" s="4">
-        <v>79.5</v>
+        <v>19</v>
       </c>
       <c r="VK35" s="4">
-        <v>48.1</v>
+        <v>32.5</v>
       </c>
       <c r="VL35" s="4">
-        <v>59.5</v>
+        <v>27</v>
       </c>
       <c r="VM35" s="4">
-        <v>53.2</v>
+        <v>57.2</v>
       </c>
     </row>
     <row r="36" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A36">
-        <v>55</v>
+      <c r="A36" s="10">
+        <v>13</v>
       </c>
       <c r="B36" t="s">
         <v>80</v>
@@ -62995,25 +62996,25 @@
       <c r="VH36">
         <v>26.75</v>
       </c>
-      <c r="VI36" s="3">
-        <v>77.2</v>
+      <c r="VI36" s="6">
+        <v>12.5</v>
       </c>
       <c r="VJ36" s="4">
-        <v>94.7</v>
+        <v>71.400000000000006</v>
       </c>
       <c r="VK36" s="4">
-        <v>25</v>
+        <v>37.1</v>
       </c>
       <c r="VL36" s="4">
-        <v>57.2</v>
+        <v>42.3</v>
       </c>
       <c r="VM36" s="4">
-        <v>55.1</v>
+        <v>22.8</v>
       </c>
     </row>
     <row r="37" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A37">
-        <v>56</v>
+      <c r="A37" s="10">
+        <v>14</v>
       </c>
       <c r="B37" t="s">
         <v>81</v>
@@ -64752,25 +64753,25 @@
       <c r="VH37">
         <v>15.69</v>
       </c>
-      <c r="VI37" s="3">
-        <v>85.5</v>
+      <c r="VI37" s="5">
+        <v>43.1</v>
       </c>
       <c r="VJ37" s="4">
-        <v>85</v>
+        <v>27.8</v>
       </c>
       <c r="VK37" s="4">
-        <v>25.4</v>
+        <v>81.8</v>
       </c>
       <c r="VL37" s="4">
-        <v>61.9</v>
+        <v>34.4</v>
       </c>
       <c r="VM37" s="4">
-        <v>81.900000000000006</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="38" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A38">
-        <v>57</v>
+      <c r="A38" s="10">
+        <v>15</v>
       </c>
       <c r="B38" t="s">
         <v>82</v>
@@ -66509,25 +66510,25 @@
       <c r="VH38">
         <v>28.06</v>
       </c>
-      <c r="VI38" s="3">
-        <v>82.4</v>
+      <c r="VI38" s="5">
+        <v>42.2</v>
       </c>
       <c r="VJ38" s="4">
-        <v>100</v>
+        <v>69.900000000000006</v>
       </c>
       <c r="VK38" s="4">
-        <v>26.2</v>
+        <v>30.4</v>
       </c>
       <c r="VL38" s="4">
-        <v>56</v>
+        <v>49.8</v>
       </c>
       <c r="VM38" s="4">
-        <v>58.1</v>
+        <v>77.2</v>
       </c>
     </row>
     <row r="39" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A39">
-        <v>58</v>
+      <c r="A39" s="10">
+        <v>16</v>
       </c>
       <c r="B39" t="s">
         <v>83</v>
@@ -68266,25 +68267,25 @@
       <c r="VH39">
         <v>14.35</v>
       </c>
-      <c r="VI39" s="3">
-        <v>89.5</v>
+      <c r="VI39" s="5">
+        <v>68.599999999999994</v>
       </c>
       <c r="VJ39" s="4">
-        <v>96.6</v>
+        <v>46.9</v>
       </c>
       <c r="VK39" s="4">
-        <v>38.5</v>
+        <v>31.3</v>
       </c>
       <c r="VL39" s="4">
-        <v>60.6</v>
+        <v>45.7</v>
       </c>
       <c r="VM39" s="4">
-        <v>62.4</v>
+        <v>67.099999999999994</v>
       </c>
     </row>
     <row r="40" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="B40" t="s">
         <v>84</v>
@@ -70024,24 +70025,24 @@
         <v>20.45</v>
       </c>
       <c r="VI40" s="5">
-        <v>63.2</v>
-      </c>
-      <c r="VJ40" s="4">
-        <v>67.900000000000006</v>
-      </c>
-      <c r="VK40" s="4">
-        <v>31.5</v>
-      </c>
-      <c r="VL40" s="4">
-        <v>55.9</v>
-      </c>
-      <c r="VM40" s="4">
-        <v>61.2</v>
+        <v>45.9</v>
+      </c>
+      <c r="VJ40" s="9">
+        <v>31</v>
+      </c>
+      <c r="VK40" s="9">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="VL40" s="9">
+        <v>36.700000000000003</v>
+      </c>
+      <c r="VM40" s="9">
+        <v>70.3</v>
       </c>
     </row>
     <row r="41" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="B41" t="s">
         <v>85</v>
@@ -71779,11 +71780,26 @@
       </c>
       <c r="VH41">
         <v>19.37</v>
+      </c>
+      <c r="VI41" s="8">
+        <v>34.299999999999997</v>
+      </c>
+      <c r="VJ41" s="4">
+        <v>61.8</v>
+      </c>
+      <c r="VK41" s="4">
+        <v>82.5</v>
+      </c>
+      <c r="VL41" s="4">
+        <v>44.1</v>
+      </c>
+      <c r="VM41" s="4">
+        <v>20.8</v>
       </c>
     </row>
     <row r="42" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="B42" t="s">
         <v>86</v>
@@ -73523,24 +73539,24 @@
         <v>24.53</v>
       </c>
       <c r="VI42" s="5">
-        <v>51.7</v>
+        <v>55.6</v>
       </c>
       <c r="VJ42" s="4">
-        <v>49.6</v>
+        <v>41.8</v>
       </c>
       <c r="VK42" s="4">
-        <v>43</v>
+        <v>55.7</v>
       </c>
       <c r="VL42" s="4">
-        <v>45.1</v>
+        <v>42.3</v>
       </c>
       <c r="VM42" s="4">
-        <v>65.599999999999994</v>
+        <v>71.7</v>
       </c>
     </row>
     <row r="43" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="B43" t="s">
         <v>87</v>
@@ -75280,24 +75296,24 @@
         <v>25.15</v>
       </c>
       <c r="VI43" s="5">
-        <v>44.6</v>
+        <v>53.1</v>
       </c>
       <c r="VJ43" s="4">
-        <v>45.6</v>
+        <v>66.099999999999994</v>
       </c>
       <c r="VK43" s="4">
-        <v>35.1</v>
+        <v>42.5</v>
       </c>
       <c r="VL43" s="4">
-        <v>55.4</v>
+        <v>47</v>
       </c>
       <c r="VM43" s="4">
-        <v>52.7</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="44" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A44">
-        <v>63</v>
+      <c r="A44" s="10">
+        <v>54</v>
       </c>
       <c r="B44" t="s">
         <v>88</v>
@@ -77037,24 +77053,24 @@
         <v>17.97</v>
       </c>
       <c r="VI44" s="5">
-        <v>67.5</v>
+        <v>55.1</v>
       </c>
       <c r="VJ44" s="4">
-        <v>63.3</v>
+        <v>29.6</v>
       </c>
       <c r="VK44" s="4">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="VL44" s="4">
-        <v>43</v>
+        <v>42.6</v>
       </c>
       <c r="VM44" s="4">
-        <v>29.3</v>
+        <v>79.2</v>
       </c>
     </row>
     <row r="45" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A45">
-        <v>64</v>
+      <c r="A45" s="10">
+        <v>55</v>
       </c>
       <c r="B45" t="s">
         <v>89</v>
@@ -78793,25 +78809,25 @@
       <c r="VH45">
         <v>22.76</v>
       </c>
-      <c r="VI45" s="6">
-        <v>12.5</v>
+      <c r="VI45" s="5">
+        <v>47.4</v>
       </c>
       <c r="VJ45" s="4">
-        <v>19</v>
+        <v>36.9</v>
       </c>
       <c r="VK45" s="4">
-        <v>32.5</v>
+        <v>44.2</v>
       </c>
       <c r="VL45" s="4">
-        <v>27</v>
+        <v>33.4</v>
       </c>
       <c r="VM45" s="4">
-        <v>57.2</v>
+        <v>64.8</v>
       </c>
     </row>
     <row r="46" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A46">
-        <v>65</v>
+      <c r="A46" s="10">
+        <v>56</v>
       </c>
       <c r="B46" t="s">
         <v>90</v>
@@ -80550,25 +80566,25 @@
       <c r="VH46">
         <v>20.71</v>
       </c>
-      <c r="VI46" s="5">
-        <v>43.1</v>
+      <c r="VI46" s="6">
+        <v>36.9</v>
       </c>
       <c r="VJ46" s="4">
-        <v>71.400000000000006</v>
+        <v>14.8</v>
       </c>
       <c r="VK46" s="4">
-        <v>37.1</v>
+        <v>43.8</v>
       </c>
       <c r="VL46" s="4">
-        <v>42.3</v>
+        <v>27.1</v>
       </c>
       <c r="VM46" s="4">
-        <v>22.8</v>
+        <v>61.4</v>
       </c>
     </row>
     <row r="47" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A47">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="B47" t="s">
         <v>91</v>
@@ -82307,25 +82323,25 @@
       <c r="VH47">
         <v>22.55</v>
       </c>
-      <c r="VI47" s="5">
-        <v>42.2</v>
+      <c r="VI47" s="6">
+        <v>16.3</v>
       </c>
       <c r="VJ47" s="4">
-        <v>27.8</v>
+        <v>34.299999999999997</v>
       </c>
       <c r="VK47" s="4">
-        <v>81.8</v>
+        <v>45.8</v>
       </c>
       <c r="VL47" s="4">
-        <v>34.4</v>
+        <v>39.6</v>
       </c>
       <c r="VM47" s="4">
-        <v>54.7</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="48" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A48">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B48" t="s">
         <v>92</v>
@@ -84064,25 +84080,25 @@
       <c r="VH48">
         <v>21.28</v>
       </c>
-      <c r="VI48" s="5">
-        <v>68.599999999999994</v>
+      <c r="VI48" s="6">
+        <v>30</v>
       </c>
       <c r="VJ48" s="4">
-        <v>69.900000000000006</v>
+        <v>39.799999999999997</v>
       </c>
       <c r="VK48" s="4">
-        <v>30.4</v>
+        <v>92.3</v>
       </c>
       <c r="VL48" s="4">
-        <v>49.8</v>
+        <v>25.8</v>
       </c>
       <c r="VM48" s="4">
-        <v>77.2</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="49" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="B49" t="s">
         <v>93</v>
@@ -85821,25 +85837,25 @@
       <c r="VH49">
         <v>26.71</v>
       </c>
-      <c r="VI49" s="5">
-        <v>45.9</v>
+      <c r="VI49" s="6">
+        <v>35.9</v>
       </c>
       <c r="VJ49" s="4">
-        <v>46.9</v>
+        <v>28.8</v>
       </c>
       <c r="VK49" s="4">
-        <v>31.3</v>
+        <v>41.7</v>
       </c>
       <c r="VL49" s="4">
-        <v>45.7</v>
+        <v>48.5</v>
       </c>
       <c r="VM49" s="4">
-        <v>67.099999999999994</v>
+        <v>69.5</v>
       </c>
     </row>
     <row r="50" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A50">
-        <v>69</v>
+      <c r="A50" s="10">
+        <v>60</v>
       </c>
       <c r="B50" t="s">
         <v>94</v>
@@ -87579,24 +87595,24 @@
         <v>20.11</v>
       </c>
       <c r="VI50" s="6">
-        <v>34.299999999999997</v>
+        <v>39.9</v>
       </c>
       <c r="VJ50" s="4">
-        <v>31</v>
+        <v>38.9</v>
       </c>
       <c r="VK50" s="4">
-        <v>37.799999999999997</v>
+        <v>15.5</v>
       </c>
       <c r="VL50" s="4">
-        <v>36.700000000000003</v>
+        <v>51.3</v>
       </c>
       <c r="VM50" s="4">
-        <v>70.3</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B51" t="s">
         <v>95</v>
@@ -89336,24 +89352,24 @@
         <v>17.45</v>
       </c>
       <c r="VI51" s="5">
-        <v>55.6</v>
+        <v>41.4</v>
       </c>
       <c r="VJ51" s="4">
-        <v>61.8</v>
+        <v>15.6</v>
       </c>
       <c r="VK51" s="4">
-        <v>82.5</v>
+        <v>41.7</v>
       </c>
       <c r="VL51" s="4">
-        <v>44.1</v>
+        <v>24.1</v>
       </c>
       <c r="VM51" s="4">
-        <v>20.8</v>
+        <v>75.099999999999994</v>
       </c>
     </row>
     <row r="52" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A52">
-        <v>108</v>
+        <v>62</v>
       </c>
       <c r="B52" t="s">
         <v>97</v>
@@ -91092,25 +91108,25 @@
       <c r="VH52">
         <v>26.49</v>
       </c>
-      <c r="VI52" s="5">
-        <v>53.1</v>
+      <c r="VI52" s="6">
+        <v>20.9</v>
       </c>
       <c r="VJ52" s="4">
-        <v>41.8</v>
+        <v>8.6</v>
       </c>
       <c r="VK52" s="4">
-        <v>55.7</v>
+        <v>52.7</v>
       </c>
       <c r="VL52" s="4">
-        <v>42.3</v>
+        <v>12.7</v>
       </c>
       <c r="VM52" s="4">
-        <v>71.7</v>
+        <v>82.8</v>
       </c>
     </row>
     <row r="53" spans="1:585" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>109</v>
+        <v>63</v>
       </c>
       <c r="B53" t="s">
         <v>98</v>
@@ -92849,25 +92865,25 @@
       <c r="VH53">
         <v>31.63</v>
       </c>
-      <c r="VI53" s="5">
-        <v>55.1</v>
+      <c r="VI53" s="6">
+        <v>18.5</v>
       </c>
       <c r="VJ53" s="4">
-        <v>66.099999999999994</v>
+        <v>7.5</v>
       </c>
       <c r="VK53" s="4">
-        <v>42.5</v>
+        <v>79.099999999999994</v>
       </c>
       <c r="VL53" s="4">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="VM53" s="4">
-        <v>46.4</v>
+        <v>73.400000000000006</v>
       </c>
     </row>
     <row r="54" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A54">
-        <v>110</v>
+        <v>64</v>
       </c>
       <c r="B54" t="s">
         <v>99</v>
@@ -94606,25 +94622,25 @@
       <c r="VH54">
         <v>28.62</v>
       </c>
-      <c r="VI54" s="5">
-        <v>47.4</v>
+      <c r="VI54" s="6">
+        <v>27.7</v>
       </c>
       <c r="VJ54" s="4">
-        <v>29.6</v>
+        <v>12.6</v>
       </c>
       <c r="VK54" s="4">
-        <v>54</v>
+        <v>65.5</v>
       </c>
       <c r="VL54" s="4">
-        <v>42.6</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="VM54" s="4">
-        <v>79.2</v>
+        <v>66.900000000000006</v>
       </c>
     </row>
     <row r="55" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>111</v>
+        <v>65</v>
       </c>
       <c r="B55" t="s">
         <v>100</v>
@@ -96364,24 +96380,24 @@
         <v>24.51</v>
       </c>
       <c r="VI55" s="6">
-        <v>36.9</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="VJ55" s="4">
-        <v>36.9</v>
+        <v>0</v>
       </c>
       <c r="VK55" s="4">
-        <v>44.2</v>
+        <v>65.7</v>
       </c>
       <c r="VL55" s="4">
-        <v>33.4</v>
+        <v>0</v>
       </c>
       <c r="VM55" s="4">
-        <v>64.8</v>
+        <v>58</v>
       </c>
     </row>
     <row r="56" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="A56">
-        <v>112</v>
+      <c r="A56" s="10">
+        <v>66</v>
       </c>
       <c r="B56" t="s">
         <v>101</v>
@@ -98121,24 +98137,24 @@
         <v>17.649999999999999</v>
       </c>
       <c r="VI56" s="6">
-        <v>16.3</v>
+        <v>0</v>
       </c>
       <c r="VJ56" s="4">
-        <v>14.8</v>
+        <v>44.3</v>
       </c>
       <c r="VK56" s="4">
-        <v>43.8</v>
+        <v>55.4</v>
       </c>
       <c r="VL56" s="4">
-        <v>27.1</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="VM56" s="4">
-        <v>61.4</v>
+        <v>17.100000000000001</v>
       </c>
     </row>
     <row r="57" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>113</v>
+        <v>67</v>
       </c>
       <c r="B57" t="s">
         <v>102</v>
@@ -99878,24 +99894,24 @@
         <v>21.77</v>
       </c>
       <c r="VI57" s="6">
-        <v>30</v>
+        <v>8.9</v>
       </c>
       <c r="VJ57" s="4">
-        <v>34.299999999999997</v>
+        <v>14.2</v>
       </c>
       <c r="VK57" s="4">
-        <v>45.8</v>
+        <v>44.3</v>
       </c>
       <c r="VL57" s="4">
-        <v>39.6</v>
+        <v>1.9</v>
       </c>
       <c r="VM57" s="4">
-        <v>45.7</v>
+        <v>75.599999999999994</v>
       </c>
     </row>
     <row r="58" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A58">
-        <v>114</v>
+        <v>68</v>
       </c>
       <c r="B58" t="s">
         <v>103</v>
@@ -101635,24 +101651,24 @@
         <v>21.95</v>
       </c>
       <c r="VI58" s="6">
-        <v>35.9</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="VJ58" s="4">
-        <v>39.799999999999997</v>
+        <v>10.6</v>
       </c>
       <c r="VK58" s="4">
-        <v>92.3</v>
+        <v>46.8</v>
       </c>
       <c r="VL58" s="4">
-        <v>25.8</v>
+        <v>16.100000000000001</v>
       </c>
       <c r="VM58" s="4">
-        <v>22.9</v>
+        <v>73.599999999999994</v>
       </c>
     </row>
     <row r="59" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="B59" t="s">
         <v>104</v>
@@ -103386,24 +103402,24 @@
         <v>22.28</v>
       </c>
       <c r="VI59" s="6">
-        <v>39.9</v>
+        <v>14.8</v>
       </c>
       <c r="VJ59" s="4">
-        <v>28.8</v>
+        <v>55</v>
       </c>
       <c r="VK59" s="4">
-        <v>41.7</v>
+        <v>41.4</v>
       </c>
       <c r="VL59" s="4">
-        <v>48.5</v>
+        <v>99.7</v>
       </c>
       <c r="VM59" s="4">
-        <v>69.5</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="60" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>117</v>
+        <v>70</v>
       </c>
       <c r="B60" t="s">
         <v>105</v>
@@ -105137,24 +105153,24 @@
         <v>27.62</v>
       </c>
       <c r="VI60" s="5">
-        <v>41.4</v>
+        <v>58.3</v>
       </c>
       <c r="VJ60" s="4">
-        <v>38.9</v>
+        <v>78.599999999999994</v>
       </c>
       <c r="VK60" s="4">
-        <v>15.5</v>
+        <v>80.7</v>
       </c>
       <c r="VL60" s="4">
-        <v>51.3</v>
+        <v>100</v>
       </c>
       <c r="VM60" s="4">
-        <v>78</v>
+        <v>14</v>
       </c>
     </row>
     <row r="61" spans="1:585" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>118</v>
+        <v>99</v>
       </c>
       <c r="B61" t="s">
         <v>106</v>
@@ -106887,38 +106903,28 @@
       <c r="VH61">
         <v>14.94</v>
       </c>
-      <c r="VI61" s="6">
-        <v>20.9</v>
+      <c r="VI61" s="3">
+        <v>91.5</v>
       </c>
       <c r="VJ61" s="4">
-        <v>15.6</v>
+        <v>96.9</v>
       </c>
       <c r="VK61" s="4">
-        <v>41.7</v>
+        <v>34.200000000000003</v>
       </c>
       <c r="VL61" s="4">
-        <v>24.1</v>
+        <v>97.5</v>
       </c>
       <c r="VM61" s="4">
-        <v>75.099999999999994</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:585" x14ac:dyDescent="0.3">
-      <c r="VI62" s="3">
-        <v>76.900000000000006</v>
-      </c>
-      <c r="VJ62" s="4">
-        <v>96.9</v>
-      </c>
-      <c r="VK62" s="4">
-        <v>34.200000000000003</v>
-      </c>
-      <c r="VL62" s="4">
-        <v>97.5</v>
-      </c>
-      <c r="VM62" s="4">
-        <v>0</v>
-      </c>
+      <c r="VI62" s="3"/>
+      <c r="VJ62" s="4"/>
+      <c r="VK62" s="4"/>
+      <c r="VL62" s="4"/>
+      <c r="VM62" s="4"/>
     </row>
     <row r="65" spans="3:251" x14ac:dyDescent="0.3">
       <c r="C65" t="s">
@@ -107678,14 +107684,11 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A3">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  <conditionalFormatting sqref="B12:B18">
+    <cfRule type="duplicateValues" dxfId="2" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A12:B18">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A19:B61">
-    <cfRule type="duplicateValues" dxfId="1" priority="6"/>
+  <conditionalFormatting sqref="B19:B61">
+    <cfRule type="duplicateValues" dxfId="1" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B62:B1048576 B1:B3 D1:D1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="5"/>

</xml_diff>